<commit_message>
Update US Open live tracker
</commit_message>
<xml_diff>
--- a/major-pool-2026-golf-analysis/us_open_player_live_tracker_2026.xlsx
+++ b/major-pool-2026-golf-analysis/us_open_player_live_tracker_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f48d3ac1ac4b44e9/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f48d3ac1ac4b44e9/Desktop/Personal Work/Data-Analyst-Portfolio/major-pool-2026-golf-analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D7D6177-66DB-47E6-8F69-7E4904CC3BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{7D7D6177-66DB-47E6-8F69-7E4904CC3BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5510287C-CB83-49EB-A954-F86633A6222F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="676">
   <si>
     <t>Player</t>
   </si>
@@ -1973,9 +1973,6 @@
   </si>
   <si>
     <t>Manual Notes</t>
-  </si>
-  <si>
-    <t>Enter Player Name</t>
   </si>
   <si>
     <t>Lineup</t>
@@ -2482,37 +2479,10 @@
     <xf numFmtId="0" fontId="11" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2530,23 +2500,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7664,16 +7661,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="8.25" customHeight="1">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="58" t="s">
         <v>548</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
@@ -7692,16 +7689,16 @@
       <c r="X1" s="2"/>
     </row>
     <row r="2" spans="1:24" ht="14.5">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="59" t="s">
         <v>549</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -7793,12 +7790,12 @@
       <c r="E5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="41" t="str">
+      <c r="F5" s="60" t="str">
         <f>IFERROR(INDEX('Master Data'!$M$2:$M$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>Best Tier 5 survival pick</v>
       </c>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -8047,16 +8044,16 @@
       <c r="A13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="39" t="str">
+      <c r="B13" s="53" t="str">
         <f>IFERROR(INDEX('Master Data'!$R$2:$R$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>T25 at Shinnecock in 2018</v>
       </c>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
+      <c r="C13" s="53"/>
+      <c r="D13" s="53"/>
+      <c r="E13" s="53"/>
+      <c r="F13" s="53"/>
+      <c r="G13" s="53"/>
+      <c r="H13" s="53"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
@@ -8076,13 +8073,13 @@
     </row>
     <row r="14" spans="1:24" ht="9.5" customHeight="1">
       <c r="A14" s="2"/>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
+      <c r="B14" s="53"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="53"/>
+      <c r="H14" s="53"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -8130,16 +8127,16 @@
       <c r="A16" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="39" t="str">
+      <c r="B16" s="53" t="str">
         <f>IFERROR(INDEX('Master Data'!$S$2:$S$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>Veteran, wind control, difficult-course comfort</v>
       </c>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
+      <c r="C16" s="53"/>
+      <c r="D16" s="53"/>
+      <c r="E16" s="53"/>
+      <c r="F16" s="53"/>
+      <c r="G16" s="53"/>
+      <c r="H16" s="53"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
@@ -8159,13 +8156,13 @@
     </row>
     <row r="17" spans="1:24" ht="9.5" customHeight="1">
       <c r="A17" s="2"/>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
@@ -8213,16 +8210,16 @@
       <c r="A19" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="42" t="str">
+      <c r="B19" s="54" t="str">
         <f>IFERROR(INDEX('Master Data'!$T$2:$T$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>Can grind pars when scoring gets ugly</v>
       </c>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="54"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="54"/>
+      <c r="G19" s="54"/>
+      <c r="H19" s="54"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -8242,13 +8239,13 @@
     </row>
     <row r="20" spans="1:24" ht="9.5" customHeight="1">
       <c r="A20" s="2"/>
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -8268,13 +8265,13 @@
     </row>
     <row r="21" spans="1:24" ht="9.5" customHeight="1">
       <c r="A21" s="2"/>
-      <c r="B21" s="42"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -8322,16 +8319,16 @@
       <c r="A23" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="43" t="str">
+      <c r="B23" s="55" t="str">
         <f>IFERROR(INDEX('Master Data'!$U$2:$U$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>Lower winning ceiling than Cameron Smith</v>
       </c>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="43"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="55"/>
+      <c r="H23" s="55"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
@@ -8351,13 +8348,13 @@
     </row>
     <row r="24" spans="1:24" ht="9.5" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43"/>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="55"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -8377,13 +8374,13 @@
     </row>
     <row r="25" spans="1:24" ht="9.5" customHeight="1">
       <c r="A25" s="2"/>
-      <c r="B25" s="43"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="43"/>
+      <c r="B25" s="55"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="55"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -8431,16 +8428,16 @@
       <c r="A27" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="44" t="str">
+      <c r="B27" s="56" t="str">
         <f>IFERROR(INDEX('Master Data'!$Q$2:$Q$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>No major form collapse concern</v>
       </c>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="44"/>
+      <c r="C27" s="56"/>
+      <c r="D27" s="56"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="56"/>
+      <c r="G27" s="56"/>
+      <c r="H27" s="56"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -8460,13 +8457,13 @@
     </row>
     <row r="28" spans="1:24" ht="9.5" customHeight="1">
       <c r="A28" s="2"/>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="44"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="44"/>
+      <c r="B28" s="56"/>
+      <c r="C28" s="56"/>
+      <c r="D28" s="56"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="56"/>
+      <c r="G28" s="56"/>
+      <c r="H28" s="56"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -8486,13 +8483,13 @@
     </row>
     <row r="29" spans="1:24" ht="9.5" customHeight="1">
       <c r="A29" s="2"/>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
+      <c r="B29" s="56"/>
+      <c r="C29" s="56"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
@@ -8540,16 +8537,16 @@
       <c r="A31" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B31" s="45" t="str">
+      <c r="B31" s="57" t="str">
         <f>IFERROR(INDEX('Master Data'!$V$2:$V$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>Useful if friends chase bigger names</v>
       </c>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="45"/>
+      <c r="C31" s="57"/>
+      <c r="D31" s="57"/>
+      <c r="E31" s="57"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="57"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
@@ -8569,13 +8566,13 @@
     </row>
     <row r="32" spans="1:24" ht="9.5" customHeight="1">
       <c r="A32" s="2"/>
-      <c r="B32" s="45"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="45"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
+      <c r="B32" s="57"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="57"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="57"/>
+      <c r="H32" s="57"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
@@ -8595,13 +8592,13 @@
     </row>
     <row r="33" spans="1:24" ht="9.5" customHeight="1">
       <c r="A33" s="2"/>
-      <c r="B33" s="45"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45"/>
-      <c r="H33" s="45"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="57"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
@@ -8649,16 +8646,16 @@
       <c r="A35" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B35" s="39" t="str">
+      <c r="B35" s="53" t="str">
         <f>IFERROR(INDEX('Master Data'!$W$2:$W$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>https://www.golfdigest.com/story/us-open-2026-power-ranking-entire-field-shinnecock-hills</v>
       </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
@@ -8706,16 +8703,16 @@
       <c r="A37" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="39" t="str">
+      <c r="B37" s="53" t="str">
         <f>IFERROR(INDEX('Master Data'!$X$2:$X$46,MATCH($B$3,'Master Data'!$A$2:$A$46,0)),"")</f>
         <v>https://www.usopen.com/</v>
       </c>
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="39"/>
-      <c r="H37" s="39"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="53"/>
+      <c r="G37" s="53"/>
+      <c r="H37" s="53"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
@@ -9853,19 +9850,31 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="B13:H14"/>
+    <mergeCell ref="B16:H17"/>
     <mergeCell ref="B37:H37"/>
     <mergeCell ref="B19:H21"/>
     <mergeCell ref="B23:H25"/>
     <mergeCell ref="B27:H29"/>
     <mergeCell ref="B31:H33"/>
     <mergeCell ref="B35:H35"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="B13:H14"/>
-    <mergeCell ref="B16:H17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FAB96B11-077E-453D-9397-11F881356E59}">
+          <x14:formula1>
+            <xm:f>'Master Data'!$A$2:$A$46</xm:f>
+          </x14:formula1>
+          <xm:sqref>B3</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -9882,16 +9891,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="8.25" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="61" t="s">
         <v>552</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
@@ -10780,21 +10789,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="29.5" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="38" t="s">
         <v>623</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
     </row>
     <row r="3" spans="1:15" ht="18.5" customHeight="1">
       <c r="A3" s="16" t="s">
@@ -10803,20 +10812,20 @@
       <c r="B3" s="17" t="s">
         <v>624</v>
       </c>
-      <c r="D3" s="58" t="s">
+      <c r="D3" s="52" t="s">
         <v>625</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="52"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="52"/>
     </row>
     <row r="4" spans="1:15" ht="9.4" customHeight="1">
       <c r="A4" s="16" t="s">
@@ -10825,20 +10834,20 @@
       <c r="B4" s="17">
         <v>70</v>
       </c>
-      <c r="D4" s="59" t="s">
-        <v>674</v>
-      </c>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="60"/>
-      <c r="O4" s="60"/>
+      <c r="D4" s="47" t="s">
+        <v>673</v>
+      </c>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="48"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="48"/>
     </row>
     <row r="5" spans="1:15" ht="28">
       <c r="A5" s="16" t="s">
@@ -10847,18 +10856,18 @@
       <c r="B5" s="31" t="s">
         <v>628</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
-      <c r="I5" s="60"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="60"/>
-      <c r="L5" s="60"/>
-      <c r="M5" s="60"/>
-      <c r="N5" s="60"/>
-      <c r="O5" s="60"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
+      <c r="L5" s="48"/>
+      <c r="M5" s="48"/>
+      <c r="N5" s="48"/>
+      <c r="O5" s="48"/>
     </row>
     <row r="6" spans="1:15" ht="32" customHeight="1">
       <c r="A6" s="16" t="s">
@@ -10867,54 +10876,54 @@
       <c r="B6" s="17" t="s">
         <v>630</v>
       </c>
-      <c r="D6" s="59"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="60"/>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="36" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B7" s="37">
         <v>8</v>
       </c>
-      <c r="D7" s="56" t="s">
-        <v>676</v>
-      </c>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="57"/>
-      <c r="L7" s="57"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
+      <c r="D7" s="49" t="s">
+        <v>675</v>
+      </c>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="50"/>
+      <c r="J7" s="50"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="50"/>
+      <c r="O7" s="50"/>
     </row>
     <row r="8" spans="1:15">
-      <c r="D8" s="59"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="61"/>
-      <c r="N8" s="61"/>
-      <c r="O8" s="61"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
+      <c r="J8" s="51"/>
+      <c r="K8" s="51"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="51"/>
+      <c r="N8" s="51"/>
+      <c r="O8" s="51"/>
     </row>
     <row r="9" spans="1:15" ht="9.75" customHeight="1">
       <c r="A9" s="15" t="s">
@@ -10968,23 +10977,25 @@
         <v>1</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>645</v>
-      </c>
-      <c r="C10" s="32"/>
+        <v>98</v>
+      </c>
+      <c r="C10" s="32">
+        <v>68</v>
+      </c>
       <c r="D10" s="32"/>
       <c r="E10" s="32"/>
       <c r="F10" s="32"/>
       <c r="G10" s="22">
         <f>COUNT(C10:F10)</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="H10" s="22">
         <f>IF(G10=0,"",SUM(C10:F10))</f>
-        <v/>
-      </c>
-      <c r="I10" s="20" t="str">
+        <v>68</v>
+      </c>
+      <c r="I10" s="20">
         <f t="shared" ref="I10:I16" si="0">IF(G10=0,"",H10-($B$4*G10))</f>
-        <v/>
+        <v>-2</v>
       </c>
       <c r="J10" s="18" t="str">
         <f>IF(G10&lt;2,"Need R1/R2",IF(SUM(C10:D10)-($B$4*2)&lt;=$B$7-4,"Likely safe",IF(SUM(C10:D10)-($B$4*2)&lt;=$B$7,"Cut watch","Cut danger")))</f>
@@ -10992,7 +11003,7 @@
       </c>
       <c r="K10" s="18" t="str">
         <f>IF(C10="","",IF(C10&lt;=VLOOKUP($B10,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(C10&lt;=VLOOKUP($B10,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(C10&lt;VLOOKUP($B10,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
-        <v/>
+        <v>Great / better than expected</v>
       </c>
       <c r="L10" s="18" t="str">
         <f>IF(D10="","",IF(D10&lt;=VLOOKUP($B10,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(D10&lt;=VLOOKUP($B10,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(D10&lt;VLOOKUP($B10,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
@@ -11013,23 +11024,25 @@
         <v>2</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>645</v>
-      </c>
-      <c r="C11" s="32"/>
+        <v>200</v>
+      </c>
+      <c r="C11" s="32">
+        <v>73</v>
+      </c>
       <c r="D11" s="32"/>
       <c r="E11" s="32"/>
       <c r="F11" s="32"/>
       <c r="G11" s="22">
         <f t="shared" ref="G11:G15" si="1">COUNT(C11:F11)</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="H11" s="22">
         <f t="shared" ref="H11:H15" si="2">IF(G11=0,"",SUM(C11:F11))</f>
-        <v/>
-      </c>
-      <c r="I11" s="20" t="str">
+        <v>73</v>
+      </c>
+      <c r="I11" s="20">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="J11" s="18" t="str">
         <f t="shared" ref="J11:J15" si="3">IF(G11&lt;2,"Need R1/R2",IF(SUM(C11:D11)-($B$4*2)&lt;=$B$7-4,"Likely safe",IF(SUM(C11:D11)-($B$4*2)&lt;=$B$7,"Cut watch","Cut danger")))</f>
@@ -11037,7 +11050,7 @@
       </c>
       <c r="K11" s="18" t="str">
         <f>IF(C11="","",IF(C11&lt;=VLOOKUP($B11,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(C11&lt;=VLOOKUP($B11,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(C11&lt;VLOOKUP($B11,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
-        <v/>
+        <v>Realistic score</v>
       </c>
       <c r="L11" s="18" t="str">
         <f>IF(D11="","",IF(D11&lt;=VLOOKUP($B11,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(D11&lt;=VLOOKUP($B11,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(D11&lt;VLOOKUP($B11,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
@@ -11058,23 +11071,25 @@
         <v>3</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>645</v>
-      </c>
-      <c r="C12" s="32"/>
+        <v>326</v>
+      </c>
+      <c r="C12" s="32">
+        <v>74</v>
+      </c>
       <c r="D12" s="32"/>
       <c r="E12" s="32"/>
       <c r="F12" s="32"/>
       <c r="G12" s="22">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="H12" s="22">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I12" s="20" t="str">
+        <v>74</v>
+      </c>
+      <c r="I12" s="20">
         <f t="shared" si="0"/>
-        <v/>
+        <v>4</v>
       </c>
       <c r="J12" s="18" t="str">
         <f t="shared" si="3"/>
@@ -11082,7 +11097,7 @@
       </c>
       <c r="K12" s="18" t="str">
         <f>IF(C12="","",IF(C12&lt;=VLOOKUP($B12,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(C12&lt;=VLOOKUP($B12,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(C12&lt;VLOOKUP($B12,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
-        <v/>
+        <v>Realistic score</v>
       </c>
       <c r="L12" s="18" t="str">
         <f>IF(D12="","",IF(D12&lt;=VLOOKUP($B12,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(D12&lt;=VLOOKUP($B12,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(D12&lt;VLOOKUP($B12,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
@@ -11103,23 +11118,25 @@
         <v>4</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>645</v>
-      </c>
-      <c r="C13" s="32"/>
+        <v>455</v>
+      </c>
+      <c r="C13" s="32">
+        <v>72</v>
+      </c>
       <c r="D13" s="32"/>
       <c r="E13" s="32"/>
       <c r="F13" s="32"/>
       <c r="G13" s="22">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="H13" s="22">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I13" s="20" t="str">
+        <v>72</v>
+      </c>
+      <c r="I13" s="20">
         <f t="shared" si="0"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J13" s="18" t="str">
         <f t="shared" si="3"/>
@@ -11127,7 +11144,7 @@
       </c>
       <c r="K13" s="18" t="str">
         <f>IF(C13="","",IF(C13&lt;=VLOOKUP($B13,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(C13&lt;=VLOOKUP($B13,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(C13&lt;VLOOKUP($B13,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
-        <v/>
+        <v>Realistic score</v>
       </c>
       <c r="L13" s="18" t="str">
         <f>IF(D13="","",IF(D13&lt;=VLOOKUP($B13,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(D13&lt;=VLOOKUP($B13,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(D13&lt;VLOOKUP($B13,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
@@ -11148,23 +11165,25 @@
         <v>5</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>645</v>
-      </c>
-      <c r="C14" s="32"/>
+        <v>470</v>
+      </c>
+      <c r="C14" s="32">
+        <v>74</v>
+      </c>
       <c r="D14" s="32"/>
       <c r="E14" s="32"/>
       <c r="F14" s="32"/>
       <c r="G14" s="22">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="H14" s="22">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I14" s="20" t="str">
+        <v>74</v>
+      </c>
+      <c r="I14" s="20">
         <f t="shared" si="0"/>
-        <v/>
+        <v>4</v>
       </c>
       <c r="J14" s="18" t="str">
         <f t="shared" si="3"/>
@@ -11172,7 +11191,7 @@
       </c>
       <c r="K14" s="18" t="str">
         <f>IF(C14="","",IF(C14&lt;=VLOOKUP($B14,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(C14&lt;=VLOOKUP($B14,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(C14&lt;VLOOKUP($B14,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
-        <v/>
+        <v>Realistic score</v>
       </c>
       <c r="L14" s="18" t="str">
         <f>IF(D14="","",IF(D14&lt;=VLOOKUP($B14,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(D14&lt;=VLOOKUP($B14,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(D14&lt;VLOOKUP($B14,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
@@ -11193,23 +11212,25 @@
         <v>6</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>645</v>
-      </c>
-      <c r="C15" s="32"/>
+        <v>485</v>
+      </c>
+      <c r="C15" s="32">
+        <v>69</v>
+      </c>
       <c r="D15" s="32"/>
       <c r="E15" s="32"/>
       <c r="F15" s="32"/>
       <c r="G15" s="22">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H15" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="H15" s="22">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I15" s="20" t="str">
+        <v>69</v>
+      </c>
+      <c r="I15" s="20">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="J15" s="18" t="str">
         <f t="shared" si="3"/>
@@ -11217,7 +11238,7 @@
       </c>
       <c r="K15" s="18" t="str">
         <f>IF(C15="","",IF(C15&lt;=VLOOKUP($B15,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(C15&lt;=VLOOKUP($B15,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(C15&lt;VLOOKUP($B15,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
-        <v/>
+        <v>Great / better than expected</v>
       </c>
       <c r="L15" s="18" t="str">
         <f>IF(D15="","",IF(D15&lt;=VLOOKUP($B15,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(D15&lt;=VLOOKUP($B15,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(D15&lt;VLOOKUP($B15,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
@@ -11236,7 +11257,7 @@
     <row r="16" spans="1:15" ht="28">
       <c r="A16" s="19"/>
       <c r="B16" s="19" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -11244,15 +11265,15 @@
       <c r="F16" s="19"/>
       <c r="G16" s="23">
         <f>SUM(G10:G15)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="23" t="str">
+        <v>6</v>
+      </c>
+      <c r="H16" s="23">
         <f>IF(G16=0,"",SUM(H10:H15))</f>
-        <v/>
-      </c>
-      <c r="I16" s="21" t="str">
+        <v>430</v>
+      </c>
+      <c r="I16" s="21">
         <f t="shared" si="0"/>
-        <v/>
+        <v>10</v>
       </c>
       <c r="J16" s="19" t="str">
         <f>IF(COUNT(C10:D15)&lt;12,"Cut still pending",IF(COUNTIF(J10:J15,"Cut danger")&gt;0,"One or more in danger",IF(COUNTIF(J10:J15,"Cut watch")&gt;0,"Cut watch active","All likely safe")))</f>
@@ -11265,14 +11286,14 @@
       <c r="O16" s="34"/>
     </row>
     <row r="18" spans="1:6" ht="16.5">
-      <c r="A18" s="49" t="s">
-        <v>647</v>
-      </c>
-      <c r="B18" s="50"/>
-      <c r="C18" s="50"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="51"/>
+      <c r="A18" s="40" t="s">
+        <v>646</v>
+      </c>
+      <c r="B18" s="41"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="42"/>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="24"/>
@@ -11287,50 +11308,50 @@
         <v>550</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>647</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>648</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" s="14" t="s">
         <v>649</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="E20" s="14" t="s">
         <v>650</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>651</v>
       </c>
       <c r="F20" s="27"/>
     </row>
     <row r="21" spans="1:6" ht="22" customHeight="1">
       <c r="A21" s="28" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
       <c r="B21" s="29">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C21" s="30">
         <f>IF(B21="","",B21-$B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D21" s="52" t="str">
+        <v>3</v>
+      </c>
+      <c r="D21" s="43" t="str">
         <f>IF(B21="","",IF(B21&lt;=VLOOKUP(A21,'Score Rules'!$A:$F,3,FALSE)-2,"Great / better than expected",IF(B21&lt;=VLOOKUP(A21,'Score Rules'!$A:$F,4,FALSE),"Realistic score",IF(B21&lt;VLOOKUP(A21,'Score Rules'!$A:$F,6,FALSE),"Surprising poor score","Very surprising score"))))</f>
         <v>Realistic score</v>
       </c>
-      <c r="E21" s="54" t="str">
+      <c r="E21" s="45" t="str">
         <f>IF(D21="","",IF(D21="Great / better than expected","Player is beating expected Shinnecock pace.",IF(D21="Realistic score","Normal U.S. Open survival round.",IF(D21="Surprising poor score","Worse than expected; watch cut pressure.","Major red flag for this player profile."))))</f>
         <v>Normal U.S. Open survival round.</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="D22" s="53"/>
-      <c r="E22" s="55"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="46"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="D23" s="53"/>
-      <c r="E23" s="55"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="46"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="D24" s="53"/>
-      <c r="E24" s="55"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -11401,9 +11422,22 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{08C1D90D-4F27-4552-8F6F-9407F8124645}">
+          <x14:formula1>
+            <xm:f>'Master Data'!$A$2:$A$46</xm:f>
+          </x14:formula1>
+          <xm:sqref>A21</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -11425,19 +11459,19 @@
         <v>631</v>
       </c>
       <c r="C1" s="15" t="s">
+        <v>651</v>
+      </c>
+      <c r="D1" s="15" t="s">
         <v>652</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>653</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>654</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>655</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>656</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -11460,7 +11494,7 @@
         <v>79</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -11483,7 +11517,7 @@
         <v>79</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -11506,7 +11540,7 @@
         <v>80</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -11529,7 +11563,7 @@
         <v>80</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -11552,7 +11586,7 @@
         <v>80</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -11575,7 +11609,7 @@
         <v>81</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -11598,7 +11632,7 @@
         <v>81</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28">
@@ -11621,7 +11655,7 @@
         <v>80</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -11644,7 +11678,7 @@
         <v>80</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -11667,7 +11701,7 @@
         <v>80</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -11690,7 +11724,7 @@
         <v>80</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -11713,7 +11747,7 @@
         <v>80</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -11736,7 +11770,7 @@
         <v>81</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -11759,7 +11793,7 @@
         <v>82</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -11782,7 +11816,7 @@
         <v>81</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -11805,7 +11839,7 @@
         <v>81</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -11828,7 +11862,7 @@
         <v>82</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
   </sheetData>

</xml_diff>